<commit_message>
handling black frames II
</commit_message>
<xml_diff>
--- a/data_overview_Charu.xlsx
+++ b/data_overview_Charu.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://tud365-my.sharepoint.com/personal/jkerssemakers_tudelft_nl/Documents/CD_recent/BN_CD25_Charu/analysis/CD23_Vesicles/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="52" documentId="13_ncr:1_{24EA889D-DAEC-4717-8157-A68EB77279B3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8A540DBB-E4B6-4D83-989D-C8F1E0BB64AB}"/>
+  <xr:revisionPtr revIDLastSave="100" documentId="13_ncr:1_{24EA889D-DAEC-4717-8157-A68EB77279B3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{42CCA11B-81E2-4B53-BBFB-B500C9513AA2}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,17 +16,28 @@
     <sheet name="general" sheetId="1" r:id="rId1"/>
     <sheet name="guvs" sheetId="2" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="83" uniqueCount="55">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="61" uniqueCount="20">
   <si>
     <t>run index</t>
   </si>
@@ -67,9 +78,6 @@
     <t>tif,easy guvs</t>
   </si>
   <si>
-    <t>guv_label</t>
-  </si>
-  <si>
     <t>crop</t>
   </si>
   <si>
@@ -85,119 +93,17 @@
     <t>dt(s)</t>
   </si>
   <si>
-    <t>file_20082025_CS_For Jacob.lif - R 4_Merged - C=1_roi0</t>
-  </si>
-  <si>
-    <t>file_20082025_CS_For Jacob.lif - R 4_Merged - C=1_roi1</t>
-  </si>
-  <si>
-    <t>file_20082025_CS_For Jacob.lif - R 4_Merged - C=1_roi2</t>
-  </si>
-  <si>
-    <t>file_20082025_CS_For Jacob.lif - R 4_Merged - C=1_roi3</t>
-  </si>
-  <si>
-    <t>file_20082025_CS_For Jacob.lif - R 4_Merged - C=1_roi4</t>
-  </si>
-  <si>
-    <t>file_20082025_CS_For Jacob.lif - R 4_Merged - C=1_roi5</t>
-  </si>
-  <si>
-    <t>file_20082025_CS_For Jacob.lif - R 4_Merged - C=1_roi6</t>
-  </si>
-  <si>
-    <t>file_20082025_CS_For Jacob.lif - R 4_Merged - C=1_roi7</t>
-  </si>
-  <si>
-    <t>file_20082025_CS_For Jacob.lif - R 4_Merged - C=1_roi8</t>
-  </si>
-  <si>
-    <t>file_20082025_CS_For Jacob.lif - R 4_Merged - C=1_roi9</t>
-  </si>
-  <si>
-    <t>file_20082025_CS_For Jacob.lif - R 4_Merged - C=1_roi10</t>
-  </si>
-  <si>
-    <t>file_20082025_CS_For Jacob.lif - R 4_Merged - C=1_roi11</t>
-  </si>
-  <si>
-    <t>file_20082025_CS_For Jacob.lif - R 4_Merged - C=1_roi12</t>
-  </si>
-  <si>
-    <t>file_20082025_CS_For Jacob.lif - R 4_Merged - C=1_roi13</t>
-  </si>
-  <si>
-    <t>file_20082025_CS_For Jacob.lif - R 4_Merged - C=1_roi14</t>
-  </si>
-  <si>
-    <t>file_20082025_CS_For Jacob.lif - R 4_Merged - C=1_roi15</t>
-  </si>
-  <si>
-    <t>file_20082025_CS_For Jacob.lif - R 4_Merged - C=1_roi16</t>
-  </si>
-  <si>
-    <t>file_20082025_CS_For Jacob.lif - R 4_Merged - C=1_roi17</t>
-  </si>
-  <si>
-    <t>file_20082025_CS_For Jacob.lif - R 4_Merged - C=1_roi18</t>
-  </si>
-  <si>
-    <t>file_20082025_CS_For Jacob.lif - R 4_Merged - C=1_roi19</t>
-  </si>
-  <si>
-    <t>file_20082025_CS_For Jacob.lif - R 4_Merged - C=1_roi20</t>
-  </si>
-  <si>
-    <t>file_20082025_CS_For Jacob.lif - R 4_Merged - C=1_roi21</t>
-  </si>
-  <si>
-    <t>file_20082025_CS_For Jacob.lif - R 4_Merged - C=1_roi22</t>
-  </si>
-  <si>
-    <t>file_20082025_CS_For Jacob.lif - R 4_Merged - C=1_roi23</t>
-  </si>
-  <si>
-    <t>file_20082025_CS_For Jacob.lif - R 4_Merged - C=1_roi24</t>
-  </si>
-  <si>
-    <t>file_20082025_CS_For Jacob.lif - R 4_Merged - C=1_roi25</t>
-  </si>
-  <si>
-    <t>file_20082025_CS_For Jacob.lif - R 4_Merged - C=1_roi26</t>
-  </si>
-  <si>
-    <t>file_20082025_CS_For Jacob.lif - R 4_Merged - C=1_roi27</t>
-  </si>
-  <si>
-    <t>file_20082025_CS_For Jacob.lif - R 4_Merged - C=1_roi28</t>
-  </si>
-  <si>
-    <t>file_20082025_CS_For Jacob.lif - R 4_Merged - C=1_roi29</t>
-  </si>
-  <si>
-    <t>file_20082025_CS_For Jacob.lif - R 4_Merged - C=1_roi30</t>
-  </si>
-  <si>
-    <t>file_20082025_CS_For Jacob.lif - R 4_Merged - C=1_roi31</t>
-  </si>
-  <si>
-    <t>file_20082025_CS_For Jacob.lif - R 4_Merged - C=1_roi32</t>
-  </si>
-  <si>
-    <t>file_20082025_CS_For Jacob.lif - R 4_Merged - C=1_roi33</t>
-  </si>
-  <si>
-    <t>file_20082025_CS_For Jacob.lif - R 4_Merged - C=1_roi34</t>
-  </si>
-  <si>
-    <t>merged big file</t>
+    <t>guv_id</t>
+  </si>
+  <si>
+    <t>hello</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -223,6 +129,14 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -244,7 +158,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -253,6 +167,8 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="1" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -268,6 +184,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -613,34 +533,35 @@
   <dimension ref="A1:G42"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="8.42578125" customWidth="1"/>
-    <col min="2" max="2" width="20" customWidth="1"/>
-    <col min="3" max="3" width="71" customWidth="1"/>
-    <col min="4" max="4" width="8.28515625" customWidth="1"/>
-    <col min="5" max="5" width="12.42578125" style="3" customWidth="1"/>
-    <col min="7" max="7" width="48.7109375" customWidth="1"/>
+    <col min="1" max="1" width="11.5703125" customWidth="1"/>
+    <col min="2" max="2" width="12.5703125" customWidth="1"/>
+    <col min="3" max="3" width="7.28515625" customWidth="1"/>
+    <col min="4" max="4" width="12.42578125" style="3" customWidth="1"/>
+    <col min="5" max="5" width="7.28515625" customWidth="1"/>
+    <col min="6" max="6" width="6.28515625" customWidth="1"/>
+    <col min="7" max="7" width="11" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
+      <c r="A1" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="B1" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="B1" t="s">
+      <c r="C1" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="D1" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="E1" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="C1" t="s">
-        <v>13</v>
-      </c>
-      <c r="D1" t="s">
-        <v>15</v>
-      </c>
-      <c r="E1" s="3" t="s">
+      <c r="F1" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="F1" t="s">
-        <v>18</v>
-      </c>
-      <c r="G1" t="s">
+      <c r="G1" s="4" t="s">
         <v>1</v>
       </c>
     </row>
@@ -649,19 +570,22 @@
         <v>0</v>
       </c>
       <c r="B2">
-        <v>4</v>
-      </c>
-      <c r="C2" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="D2" s="2">
-        <v>0</v>
-      </c>
-      <c r="E2" s="3">
-        <v>1000000</v>
-      </c>
-      <c r="F2">
-        <v>1</v>
+        <v>0</v>
+      </c>
+      <c r="C2" s="2">
+        <v>0</v>
+      </c>
+      <c r="D2" s="3">
+        <v>1000000</v>
+      </c>
+      <c r="E2">
+        <v>1</v>
+      </c>
+      <c r="F2" s="2">
+        <v>1</v>
+      </c>
+      <c r="G2" t="s">
+        <v>19</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
@@ -669,19 +593,22 @@
         <v>0</v>
       </c>
       <c r="B3">
-        <v>4</v>
-      </c>
-      <c r="C3" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="D3" s="2">
-        <v>0</v>
-      </c>
-      <c r="E3" s="3">
-        <v>1000000</v>
-      </c>
-      <c r="F3">
-        <v>1</v>
+        <v>0</v>
+      </c>
+      <c r="C3" s="2">
+        <v>1</v>
+      </c>
+      <c r="D3" s="3">
+        <v>1000000</v>
+      </c>
+      <c r="E3">
+        <v>1</v>
+      </c>
+      <c r="F3" s="2">
+        <v>1</v>
+      </c>
+      <c r="G3" t="s">
+        <v>19</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
@@ -689,19 +616,22 @@
         <v>0</v>
       </c>
       <c r="B4">
-        <v>4</v>
-      </c>
-      <c r="C4" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="D4" s="2">
-        <v>0</v>
-      </c>
-      <c r="E4" s="3">
-        <v>1000000</v>
-      </c>
-      <c r="F4">
-        <v>1</v>
+        <v>0</v>
+      </c>
+      <c r="C4" s="2">
+        <v>2</v>
+      </c>
+      <c r="D4" s="3">
+        <v>1000000</v>
+      </c>
+      <c r="E4">
+        <v>1</v>
+      </c>
+      <c r="F4" s="2">
+        <v>1</v>
+      </c>
+      <c r="G4" t="s">
+        <v>19</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
@@ -709,19 +639,22 @@
         <v>0</v>
       </c>
       <c r="B5">
-        <v>4</v>
-      </c>
-      <c r="C5" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="D5" s="2">
-        <v>0</v>
-      </c>
-      <c r="E5" s="3">
-        <v>1000000</v>
-      </c>
-      <c r="F5">
-        <v>1</v>
+        <v>0</v>
+      </c>
+      <c r="C5" s="2">
+        <v>3</v>
+      </c>
+      <c r="D5" s="3">
+        <v>1000000</v>
+      </c>
+      <c r="E5">
+        <v>1</v>
+      </c>
+      <c r="F5" s="2">
+        <v>1</v>
+      </c>
+      <c r="G5" t="s">
+        <v>19</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
@@ -729,19 +662,22 @@
         <v>0</v>
       </c>
       <c r="B6">
+        <v>0</v>
+      </c>
+      <c r="C6" s="2">
         <v>4</v>
       </c>
-      <c r="C6" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="D6" s="2">
-        <v>0</v>
-      </c>
-      <c r="E6" s="3">
-        <v>1000000</v>
-      </c>
-      <c r="F6">
-        <v>1</v>
+      <c r="D6" s="3">
+        <v>1000000</v>
+      </c>
+      <c r="E6">
+        <v>1</v>
+      </c>
+      <c r="F6" s="2">
+        <v>1</v>
+      </c>
+      <c r="G6" t="s">
+        <v>19</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
@@ -749,19 +685,22 @@
         <v>0</v>
       </c>
       <c r="B7">
-        <v>4</v>
-      </c>
-      <c r="C7" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="D7" s="2">
-        <v>0</v>
-      </c>
-      <c r="E7" s="3">
-        <v>1000000</v>
-      </c>
-      <c r="F7">
-        <v>1</v>
+        <v>0</v>
+      </c>
+      <c r="C7" s="2">
+        <v>5</v>
+      </c>
+      <c r="D7" s="3">
+        <v>1000000</v>
+      </c>
+      <c r="E7">
+        <v>1</v>
+      </c>
+      <c r="F7" s="2">
+        <v>1</v>
+      </c>
+      <c r="G7" t="s">
+        <v>19</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
@@ -769,19 +708,22 @@
         <v>0</v>
       </c>
       <c r="B8">
-        <v>4</v>
-      </c>
-      <c r="C8" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="D8" s="2">
-        <v>0</v>
-      </c>
-      <c r="E8" s="3">
-        <v>1000000</v>
-      </c>
-      <c r="F8">
-        <v>1</v>
+        <v>0</v>
+      </c>
+      <c r="C8" s="2">
+        <v>6</v>
+      </c>
+      <c r="D8" s="3">
+        <v>1000000</v>
+      </c>
+      <c r="E8">
+        <v>1</v>
+      </c>
+      <c r="F8" s="2">
+        <v>1</v>
+      </c>
+      <c r="G8" t="s">
+        <v>19</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
@@ -791,20 +733,20 @@
       <c r="B9">
         <v>0</v>
       </c>
-      <c r="C9" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="D9" s="2">
-        <v>1</v>
-      </c>
-      <c r="E9" s="3">
-        <v>1000000</v>
-      </c>
-      <c r="F9">
+      <c r="C9" s="2">
+        <v>7</v>
+      </c>
+      <c r="D9" s="3">
+        <v>1000000</v>
+      </c>
+      <c r="E9">
+        <v>1</v>
+      </c>
+      <c r="F9" s="2">
         <v>1</v>
       </c>
       <c r="G9" t="s">
-        <v>54</v>
+        <v>19</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
@@ -814,20 +756,20 @@
       <c r="B10">
         <v>0</v>
       </c>
-      <c r="C10" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="D10" s="2">
-        <v>1</v>
-      </c>
-      <c r="E10" s="3">
-        <v>1000000</v>
-      </c>
-      <c r="F10">
+      <c r="C10" s="2">
+        <v>8</v>
+      </c>
+      <c r="D10" s="3">
+        <v>1000000</v>
+      </c>
+      <c r="E10">
+        <v>1</v>
+      </c>
+      <c r="F10" s="2">
         <v>1</v>
       </c>
       <c r="G10" t="s">
-        <v>54</v>
+        <v>19</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
@@ -837,20 +779,20 @@
       <c r="B11">
         <v>0</v>
       </c>
-      <c r="C11" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="D11" s="2">
-        <v>1</v>
-      </c>
-      <c r="E11" s="3">
-        <v>1000000</v>
-      </c>
-      <c r="F11">
+      <c r="C11" s="2">
+        <v>9</v>
+      </c>
+      <c r="D11" s="3">
+        <v>1000000</v>
+      </c>
+      <c r="E11">
+        <v>1</v>
+      </c>
+      <c r="F11" s="2">
         <v>1</v>
       </c>
       <c r="G11" t="s">
-        <v>54</v>
+        <v>19</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
@@ -860,20 +802,20 @@
       <c r="B12">
         <v>0</v>
       </c>
-      <c r="C12" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="D12" s="2">
-        <v>1</v>
-      </c>
-      <c r="E12" s="3">
-        <v>1000000</v>
-      </c>
-      <c r="F12">
+      <c r="C12" s="2">
+        <v>10</v>
+      </c>
+      <c r="D12" s="3">
+        <v>1000000</v>
+      </c>
+      <c r="E12">
+        <v>1</v>
+      </c>
+      <c r="F12" s="2">
         <v>1</v>
       </c>
       <c r="G12" t="s">
-        <v>54</v>
+        <v>19</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
@@ -883,20 +825,20 @@
       <c r="B13">
         <v>0</v>
       </c>
-      <c r="C13" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="D13" s="2">
-        <v>1</v>
-      </c>
-      <c r="E13" s="3">
-        <v>1000000</v>
-      </c>
-      <c r="F13">
+      <c r="C13" s="2">
+        <v>11</v>
+      </c>
+      <c r="D13" s="3">
+        <v>1000000</v>
+      </c>
+      <c r="E13">
+        <v>1</v>
+      </c>
+      <c r="F13" s="2">
         <v>1</v>
       </c>
       <c r="G13" t="s">
-        <v>54</v>
+        <v>19</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">
@@ -906,20 +848,20 @@
       <c r="B14">
         <v>0</v>
       </c>
-      <c r="C14" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="D14" s="2">
-        <v>1</v>
-      </c>
-      <c r="E14" s="3">
-        <v>1000000</v>
-      </c>
-      <c r="F14">
+      <c r="C14" s="2">
+        <v>12</v>
+      </c>
+      <c r="D14" s="3">
+        <v>1000000</v>
+      </c>
+      <c r="E14">
+        <v>1</v>
+      </c>
+      <c r="F14" s="2">
         <v>1</v>
       </c>
       <c r="G14" t="s">
-        <v>54</v>
+        <v>19</v>
       </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.25">
@@ -929,20 +871,20 @@
       <c r="B15">
         <v>0</v>
       </c>
-      <c r="C15" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="D15" s="2">
-        <v>1</v>
-      </c>
-      <c r="E15" s="3">
-        <v>1000000</v>
-      </c>
-      <c r="F15">
+      <c r="C15" s="2">
+        <v>13</v>
+      </c>
+      <c r="D15" s="3">
+        <v>1000000</v>
+      </c>
+      <c r="E15">
+        <v>1</v>
+      </c>
+      <c r="F15" s="2">
         <v>1</v>
       </c>
       <c r="G15" t="s">
-        <v>54</v>
+        <v>19</v>
       </c>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.25">
@@ -952,20 +894,20 @@
       <c r="B16">
         <v>0</v>
       </c>
-      <c r="C16" s="2" t="s">
-        <v>33</v>
-      </c>
-      <c r="D16" s="2">
-        <v>1</v>
-      </c>
-      <c r="E16" s="3">
-        <v>1000000</v>
-      </c>
-      <c r="F16">
+      <c r="C16" s="2">
+        <v>14</v>
+      </c>
+      <c r="D16" s="3">
+        <v>1000000</v>
+      </c>
+      <c r="E16">
+        <v>1</v>
+      </c>
+      <c r="F16" s="2">
         <v>1</v>
       </c>
       <c r="G16" t="s">
-        <v>54</v>
+        <v>19</v>
       </c>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.25">
@@ -975,20 +917,20 @@
       <c r="B17">
         <v>0</v>
       </c>
-      <c r="C17" s="2" t="s">
-        <v>34</v>
-      </c>
-      <c r="D17" s="2">
-        <v>1</v>
-      </c>
-      <c r="E17" s="3">
-        <v>1000000</v>
-      </c>
-      <c r="F17">
+      <c r="C17" s="2">
+        <v>15</v>
+      </c>
+      <c r="D17" s="3">
+        <v>1000000</v>
+      </c>
+      <c r="E17">
+        <v>1</v>
+      </c>
+      <c r="F17" s="2">
         <v>1</v>
       </c>
       <c r="G17" t="s">
-        <v>54</v>
+        <v>19</v>
       </c>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.25">
@@ -998,20 +940,20 @@
       <c r="B18">
         <v>0</v>
       </c>
-      <c r="C18" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="D18" s="2">
-        <v>1</v>
-      </c>
-      <c r="E18" s="3">
-        <v>1000000</v>
-      </c>
-      <c r="F18">
+      <c r="C18" s="2">
+        <v>16</v>
+      </c>
+      <c r="D18" s="3">
+        <v>1000000</v>
+      </c>
+      <c r="E18">
+        <v>1</v>
+      </c>
+      <c r="F18" s="2">
         <v>1</v>
       </c>
       <c r="G18" t="s">
-        <v>54</v>
+        <v>19</v>
       </c>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.25">
@@ -1021,20 +963,20 @@
       <c r="B19">
         <v>0</v>
       </c>
-      <c r="C19" s="2" t="s">
-        <v>36</v>
-      </c>
-      <c r="D19" s="2">
-        <v>1</v>
-      </c>
-      <c r="E19" s="3">
-        <v>1000000</v>
-      </c>
-      <c r="F19">
+      <c r="C19" s="2">
+        <v>17</v>
+      </c>
+      <c r="D19" s="3">
+        <v>1000000</v>
+      </c>
+      <c r="E19">
+        <v>1</v>
+      </c>
+      <c r="F19" s="2">
         <v>1</v>
       </c>
       <c r="G19" t="s">
-        <v>54</v>
+        <v>19</v>
       </c>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.25">
@@ -1044,20 +986,20 @@
       <c r="B20">
         <v>0</v>
       </c>
-      <c r="C20" s="2" t="s">
-        <v>37</v>
-      </c>
-      <c r="D20" s="2">
-        <v>1</v>
-      </c>
-      <c r="E20" s="3">
-        <v>1000000</v>
-      </c>
-      <c r="F20">
+      <c r="C20" s="2">
+        <v>18</v>
+      </c>
+      <c r="D20" s="3">
+        <v>1000000</v>
+      </c>
+      <c r="E20">
+        <v>1</v>
+      </c>
+      <c r="F20" s="2">
         <v>1</v>
       </c>
       <c r="G20" t="s">
-        <v>54</v>
+        <v>19</v>
       </c>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.25">
@@ -1067,20 +1009,20 @@
       <c r="B21">
         <v>0</v>
       </c>
-      <c r="C21" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="D21" s="2">
-        <v>1</v>
-      </c>
-      <c r="E21" s="3">
-        <v>1000000</v>
-      </c>
-      <c r="F21">
+      <c r="C21" s="2">
+        <v>19</v>
+      </c>
+      <c r="D21" s="3">
+        <v>1000000</v>
+      </c>
+      <c r="E21">
+        <v>1</v>
+      </c>
+      <c r="F21" s="2">
         <v>1</v>
       </c>
       <c r="G21" t="s">
-        <v>54</v>
+        <v>19</v>
       </c>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.25">
@@ -1090,20 +1032,20 @@
       <c r="B22">
         <v>0</v>
       </c>
-      <c r="C22" s="2" t="s">
-        <v>39</v>
-      </c>
-      <c r="D22" s="2">
-        <v>1</v>
-      </c>
-      <c r="E22" s="3">
-        <v>1000000</v>
-      </c>
-      <c r="F22">
+      <c r="C22" s="2">
+        <v>20</v>
+      </c>
+      <c r="D22" s="3">
+        <v>1000000</v>
+      </c>
+      <c r="E22">
+        <v>1</v>
+      </c>
+      <c r="F22" s="2">
         <v>1</v>
       </c>
       <c r="G22" t="s">
-        <v>54</v>
+        <v>19</v>
       </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.25">
@@ -1113,20 +1055,20 @@
       <c r="B23">
         <v>0</v>
       </c>
-      <c r="C23" s="2" t="s">
-        <v>40</v>
-      </c>
-      <c r="D23" s="2">
-        <v>1</v>
-      </c>
-      <c r="E23" s="3">
-        <v>1000000</v>
-      </c>
-      <c r="F23">
+      <c r="C23" s="2">
+        <v>21</v>
+      </c>
+      <c r="D23" s="3">
+        <v>1000000</v>
+      </c>
+      <c r="E23">
+        <v>1</v>
+      </c>
+      <c r="F23" s="2">
         <v>1</v>
       </c>
       <c r="G23" t="s">
-        <v>54</v>
+        <v>19</v>
       </c>
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.25">
@@ -1136,20 +1078,20 @@
       <c r="B24">
         <v>0</v>
       </c>
-      <c r="C24" s="2" t="s">
-        <v>41</v>
-      </c>
-      <c r="D24" s="2">
-        <v>1</v>
-      </c>
-      <c r="E24" s="3">
-        <v>1000000</v>
-      </c>
-      <c r="F24">
+      <c r="C24" s="2">
+        <v>22</v>
+      </c>
+      <c r="D24" s="3">
+        <v>1000000</v>
+      </c>
+      <c r="E24">
+        <v>1</v>
+      </c>
+      <c r="F24" s="2">
         <v>1</v>
       </c>
       <c r="G24" t="s">
-        <v>54</v>
+        <v>19</v>
       </c>
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.25">
@@ -1159,20 +1101,20 @@
       <c r="B25">
         <v>0</v>
       </c>
-      <c r="C25" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="D25" s="2">
-        <v>1</v>
-      </c>
-      <c r="E25" s="3">
-        <v>1000000</v>
-      </c>
-      <c r="F25">
+      <c r="C25" s="2">
+        <v>23</v>
+      </c>
+      <c r="D25" s="3">
+        <v>1000000</v>
+      </c>
+      <c r="E25">
+        <v>1</v>
+      </c>
+      <c r="F25" s="2">
         <v>1</v>
       </c>
       <c r="G25" t="s">
-        <v>54</v>
+        <v>19</v>
       </c>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.25">
@@ -1182,20 +1124,20 @@
       <c r="B26">
         <v>0</v>
       </c>
-      <c r="C26" s="2" t="s">
-        <v>43</v>
-      </c>
-      <c r="D26" s="2">
-        <v>1</v>
-      </c>
-      <c r="E26" s="3">
-        <v>1000000</v>
-      </c>
-      <c r="F26">
+      <c r="C26" s="2">
+        <v>24</v>
+      </c>
+      <c r="D26" s="3">
+        <v>1000000</v>
+      </c>
+      <c r="E26">
+        <v>1</v>
+      </c>
+      <c r="F26" s="2">
         <v>1</v>
       </c>
       <c r="G26" t="s">
-        <v>54</v>
+        <v>19</v>
       </c>
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.25">
@@ -1205,20 +1147,20 @@
       <c r="B27">
         <v>0</v>
       </c>
-      <c r="C27" s="2" t="s">
-        <v>44</v>
-      </c>
-      <c r="D27" s="2">
-        <v>1</v>
-      </c>
-      <c r="E27" s="3">
-        <v>1000000</v>
-      </c>
-      <c r="F27">
+      <c r="C27" s="2">
+        <v>25</v>
+      </c>
+      <c r="D27" s="3">
+        <v>1000000</v>
+      </c>
+      <c r="E27">
+        <v>1</v>
+      </c>
+      <c r="F27" s="2">
         <v>1</v>
       </c>
       <c r="G27" t="s">
-        <v>54</v>
+        <v>19</v>
       </c>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.25">
@@ -1228,20 +1170,20 @@
       <c r="B28">
         <v>0</v>
       </c>
-      <c r="C28" s="2" t="s">
-        <v>45</v>
-      </c>
-      <c r="D28" s="2">
-        <v>1</v>
-      </c>
-      <c r="E28" s="3">
-        <v>1000000</v>
-      </c>
-      <c r="F28">
+      <c r="C28" s="2">
+        <v>26</v>
+      </c>
+      <c r="D28" s="3">
+        <v>1000000</v>
+      </c>
+      <c r="E28">
+        <v>1</v>
+      </c>
+      <c r="F28" s="2">
         <v>1</v>
       </c>
       <c r="G28" t="s">
-        <v>54</v>
+        <v>19</v>
       </c>
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.25">
@@ -1251,20 +1193,20 @@
       <c r="B29">
         <v>0</v>
       </c>
-      <c r="C29" s="2" t="s">
-        <v>46</v>
-      </c>
-      <c r="D29" s="2">
-        <v>1</v>
-      </c>
-      <c r="E29" s="3">
-        <v>1000000</v>
-      </c>
-      <c r="F29">
+      <c r="C29" s="2">
+        <v>27</v>
+      </c>
+      <c r="D29" s="3">
+        <v>1000000</v>
+      </c>
+      <c r="E29">
+        <v>1</v>
+      </c>
+      <c r="F29" s="2">
         <v>1</v>
       </c>
       <c r="G29" t="s">
-        <v>54</v>
+        <v>19</v>
       </c>
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.25">
@@ -1274,20 +1216,20 @@
       <c r="B30">
         <v>0</v>
       </c>
-      <c r="C30" s="2" t="s">
-        <v>47</v>
-      </c>
-      <c r="D30" s="2">
-        <v>1</v>
-      </c>
-      <c r="E30" s="3">
-        <v>1000000</v>
-      </c>
-      <c r="F30">
+      <c r="C30" s="2">
+        <v>28</v>
+      </c>
+      <c r="D30" s="3">
+        <v>1000000</v>
+      </c>
+      <c r="E30">
+        <v>1</v>
+      </c>
+      <c r="F30" s="2">
         <v>1</v>
       </c>
       <c r="G30" t="s">
-        <v>54</v>
+        <v>19</v>
       </c>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.25">
@@ -1297,20 +1239,20 @@
       <c r="B31">
         <v>0</v>
       </c>
-      <c r="C31" s="2" t="s">
-        <v>48</v>
-      </c>
-      <c r="D31" s="2">
-        <v>1</v>
-      </c>
-      <c r="E31" s="3">
-        <v>1000000</v>
-      </c>
-      <c r="F31">
+      <c r="C31" s="2">
+        <v>29</v>
+      </c>
+      <c r="D31" s="3">
+        <v>1000000</v>
+      </c>
+      <c r="E31">
+        <v>1</v>
+      </c>
+      <c r="F31" s="2">
         <v>1</v>
       </c>
       <c r="G31" t="s">
-        <v>54</v>
+        <v>19</v>
       </c>
     </row>
     <row r="32" spans="1:7" x14ac:dyDescent="0.25">
@@ -1320,20 +1262,20 @@
       <c r="B32">
         <v>0</v>
       </c>
-      <c r="C32" s="2" t="s">
-        <v>49</v>
-      </c>
-      <c r="D32" s="2">
-        <v>1</v>
-      </c>
-      <c r="E32" s="3">
-        <v>1000000</v>
-      </c>
-      <c r="F32">
+      <c r="C32" s="2">
+        <v>30</v>
+      </c>
+      <c r="D32" s="3">
+        <v>1000000</v>
+      </c>
+      <c r="E32">
+        <v>1</v>
+      </c>
+      <c r="F32" s="2">
         <v>1</v>
       </c>
       <c r="G32" t="s">
-        <v>54</v>
+        <v>19</v>
       </c>
     </row>
     <row r="33" spans="1:7" x14ac:dyDescent="0.25">
@@ -1343,20 +1285,20 @@
       <c r="B33">
         <v>0</v>
       </c>
-      <c r="C33" s="2" t="s">
-        <v>50</v>
-      </c>
-      <c r="D33" s="2">
-        <v>1</v>
-      </c>
-      <c r="E33" s="3">
-        <v>1000000</v>
-      </c>
-      <c r="F33">
+      <c r="C33" s="2">
+        <v>31</v>
+      </c>
+      <c r="D33" s="3">
+        <v>1000000</v>
+      </c>
+      <c r="E33">
+        <v>1</v>
+      </c>
+      <c r="F33" s="2">
         <v>1</v>
       </c>
       <c r="G33" t="s">
-        <v>54</v>
+        <v>19</v>
       </c>
     </row>
     <row r="34" spans="1:7" x14ac:dyDescent="0.25">
@@ -1366,20 +1308,20 @@
       <c r="B34">
         <v>0</v>
       </c>
-      <c r="C34" s="2" t="s">
-        <v>51</v>
-      </c>
-      <c r="D34" s="2">
-        <v>1</v>
-      </c>
-      <c r="E34" s="3">
-        <v>1000000</v>
-      </c>
-      <c r="F34">
+      <c r="C34" s="2">
+        <v>32</v>
+      </c>
+      <c r="D34" s="3">
+        <v>1000000</v>
+      </c>
+      <c r="E34">
+        <v>1</v>
+      </c>
+      <c r="F34" s="2">
         <v>1</v>
       </c>
       <c r="G34" t="s">
-        <v>54</v>
+        <v>19</v>
       </c>
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.25">
@@ -1389,20 +1331,20 @@
       <c r="B35">
         <v>0</v>
       </c>
-      <c r="C35" s="2" t="s">
-        <v>52</v>
-      </c>
-      <c r="D35" s="2">
-        <v>1</v>
-      </c>
-      <c r="E35" s="3">
-        <v>1000000</v>
-      </c>
-      <c r="F35">
+      <c r="C35" s="2">
+        <v>33</v>
+      </c>
+      <c r="D35" s="3">
+        <v>1000000</v>
+      </c>
+      <c r="E35">
+        <v>1</v>
+      </c>
+      <c r="F35" s="2">
         <v>1</v>
       </c>
       <c r="G35" t="s">
-        <v>54</v>
+        <v>19</v>
       </c>
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.25">
@@ -1412,48 +1354,163 @@
       <c r="B36">
         <v>0</v>
       </c>
-      <c r="C36" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="D36" s="2">
-        <v>1</v>
-      </c>
-      <c r="E36" s="3">
-        <v>1000000</v>
-      </c>
-      <c r="F36">
+      <c r="C36" s="2">
+        <v>34</v>
+      </c>
+      <c r="D36" s="3">
+        <v>1000000</v>
+      </c>
+      <c r="E36">
+        <v>1</v>
+      </c>
+      <c r="F36" s="2">
         <v>1</v>
       </c>
       <c r="G36" t="s">
-        <v>54</v>
+        <v>19</v>
       </c>
     </row>
     <row r="37" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="C37" s="2"/>
-      <c r="D37" s="2"/>
+      <c r="A37">
+        <v>0</v>
+      </c>
+      <c r="B37">
+        <v>1</v>
+      </c>
+      <c r="C37" s="2">
+        <v>0</v>
+      </c>
+      <c r="D37" s="3">
+        <v>1000000</v>
+      </c>
+      <c r="E37">
+        <v>1</v>
+      </c>
+      <c r="F37" s="2">
+        <v>1</v>
+      </c>
+      <c r="G37" t="s">
+        <v>19</v>
+      </c>
     </row>
     <row r="38" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="C38" s="2"/>
-      <c r="D38" s="2"/>
+      <c r="A38">
+        <v>0</v>
+      </c>
+      <c r="B38">
+        <v>1</v>
+      </c>
+      <c r="C38" s="2">
+        <v>1</v>
+      </c>
+      <c r="D38" s="3">
+        <v>1000000</v>
+      </c>
+      <c r="E38">
+        <v>1</v>
+      </c>
+      <c r="F38" s="2">
+        <v>1</v>
+      </c>
+      <c r="G38" t="s">
+        <v>19</v>
+      </c>
     </row>
     <row r="39" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="C39" s="2"/>
-      <c r="D39" s="2"/>
+      <c r="A39">
+        <v>0</v>
+      </c>
+      <c r="B39">
+        <v>1</v>
+      </c>
+      <c r="C39" s="2">
+        <v>2</v>
+      </c>
+      <c r="D39" s="3">
+        <v>1000000</v>
+      </c>
+      <c r="E39">
+        <v>1</v>
+      </c>
+      <c r="F39" s="2">
+        <v>1</v>
+      </c>
+      <c r="G39" t="s">
+        <v>19</v>
+      </c>
     </row>
     <row r="40" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="C40" s="2"/>
-      <c r="D40" s="2"/>
+      <c r="A40">
+        <v>0</v>
+      </c>
+      <c r="B40">
+        <v>1</v>
+      </c>
+      <c r="C40" s="2">
+        <v>3</v>
+      </c>
+      <c r="D40" s="3">
+        <v>1000000</v>
+      </c>
+      <c r="E40">
+        <v>1</v>
+      </c>
+      <c r="F40" s="2">
+        <v>1</v>
+      </c>
+      <c r="G40" t="s">
+        <v>19</v>
+      </c>
     </row>
     <row r="41" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="C41" s="2"/>
-      <c r="D41" s="2"/>
+      <c r="A41">
+        <v>0</v>
+      </c>
+      <c r="B41">
+        <v>1</v>
+      </c>
+      <c r="C41" s="2">
+        <v>4</v>
+      </c>
+      <c r="D41" s="3">
+        <v>1000000</v>
+      </c>
+      <c r="E41">
+        <v>1</v>
+      </c>
+      <c r="F41" s="2">
+        <v>1</v>
+      </c>
+      <c r="G41" t="s">
+        <v>19</v>
+      </c>
     </row>
     <row r="42" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="C42" s="2"/>
-      <c r="D42" s="2"/>
+      <c r="A42">
+        <v>0</v>
+      </c>
+      <c r="B42">
+        <v>1</v>
+      </c>
+      <c r="C42" s="2">
+        <v>5</v>
+      </c>
+      <c r="D42" s="3">
+        <v>1000000</v>
+      </c>
+      <c r="E42">
+        <v>1</v>
+      </c>
+      <c r="F42" s="2">
+        <v>1</v>
+      </c>
+      <c r="G42" t="s">
+        <v>19</v>
+      </c>
     </row>
   </sheetData>
   <phoneticPr fontId="3" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>